<commit_message>
feat: function added to save image on helpers
</commit_message>
<xml_diff>
--- a/internal/stock_movements/files/product_master_lists.xlsx
+++ b/internal/stock_movements/files/product_master_lists.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MY CODES\rdev-go-api\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MY CODES\rdev-go-api\internal\stock_movements\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C0A6DD-283A-43EB-9AA9-4380826E92BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B5F89F4-060E-4930-BCF7-44D54D593909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4545" yWindow="5535" windowWidth="28800" windowHeight="15885" xr2:uid="{0D04EA74-2CBB-4A1C-B34C-B69E562D4DAB}"/>
   </bookViews>
@@ -38,8 +38,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="63">
   <si>
     <t>SKU</t>
   </si>
@@ -225,6 +247,9 @@
   </si>
   <si>
     <t>AP-D39</t>
+  </si>
+  <si>
+    <t>Product Image</t>
   </si>
 </sst>
 </file>
@@ -278,6 +303,72 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+    <v>Bread on a pan</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+    <k n="Text" t="s"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -597,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B2EFC18-89EB-48BB-87FD-4A8084BB07CC}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -609,7 +700,7 @@
     <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -631,8 +722,11 @@
       <c r="G1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -651,8 +745,11 @@
       <c r="G2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>61</v>
       </c>
@@ -675,7 +772,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -695,7 +792,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -715,7 +812,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -735,7 +832,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -755,7 +852,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -775,7 +872,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -795,7 +892,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -815,7 +912,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -835,7 +932,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -855,7 +952,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -875,7 +972,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -895,7 +992,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -915,7 +1012,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>29</v>
       </c>

</xml_diff>